<commit_message>
Error checking for incomplete data
</commit_message>
<xml_diff>
--- a/MemberListTemplate.xlsx
+++ b/MemberListTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASCC\Desktop\driverclusters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF2000D-53AA-433B-9EAE-EEA49A3E0BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6A5325C-BB1A-4145-90EB-6C68D194E1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="390" windowWidth="28800" windowHeight="15090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="First" sheetId="1" r:id="rId1"/>

</xml_diff>